<commit_message>
fild upload 기능 구현  - download 미구현 (구현중..)
</commit_message>
<xml_diff>
--- a/src/main/resources/doc/PONKIDS-테이블정의서_v2.5.xlsx
+++ b/src/main/resources/doc/PONKIDS-테이블정의서_v2.5.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\git\ponkids\src\main\resources\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E8276AE-91DB-4DC9-B6A8-03B2DB6BF3ED}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{820E7562-9D4C-4DE2-8A61-E0741416B130}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="855" windowWidth="28800" windowHeight="11475" tabRatio="777" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32960,10 +32960,7 @@
       <c r="S327" s="109" t="s">
         <v>406</v>
       </c>
-      <c r="T327" s="132" t="str">
-        <f>"SEQ_"&amp;D327&amp;"_SEQ"</f>
-        <v>SEQ_TB_ATCH_FILE_DETAIL_SEQ</v>
-      </c>
+      <c r="T327" s="132"/>
       <c r="U327" s="132"/>
       <c r="V327" s="109"/>
       <c r="W327" s="90"/>
@@ -32982,11 +32979,11 @@
       </c>
       <c r="AB327" s="50" t="str">
         <f t="shared" si="58"/>
-        <v>CREATE SEQUENCE SEQ_TB_ATCH_FILE_DETAIL_SEQ START 100000;</v>
+        <v/>
       </c>
       <c r="AC327" s="50" t="str">
         <f t="shared" si="81"/>
-        <v>ALTER TABLE TB_ATCH_FILE_DETAIL ALTER COLUMN FILE_SEQ SET DEFAULT NEXTVAL('SEQ_TB_ATCH_FILE_DETAIL_SEQ');</v>
+        <v/>
       </c>
       <c r="AD327" s="50" t="str">
         <f t="shared" si="83"/>

</xml_diff>